<commit_message>
Update repository to match latest manuscript materials
</commit_message>
<xml_diff>
--- a/data/decontamination/phylogenomic_sets/posthoc_audit_GS-Zhang2025-B.xlsx
+++ b/data/decontamination/phylogenomic_sets/posthoc_audit_GS-Zhang2025-B.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linweili/Important_files/课题进展/Nature_submission_rechecked_precise_red/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linweili/Important_files/课题进展/Nature_submission_0803/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1284ED8A-D903-0E4F-9873-6B1E2963F3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6FD834-1729-8C40-AA26-554D5E7600F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="17660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -55,16 +55,16 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Supplementary Table 7 | Contamination categories identified in the independent post hoc audit</t>
-  </si>
-  <si>
     <t>Additional contamination in post hoc audit (%)</t>
   </si>
   <si>
-    <t>Percentages are calculated on a contig-weighted basis. Additional contamination categories represent source-resolved contamination identified during the post hoc audit after primary decontamination.</t>
-  </si>
-  <si>
     <t>Eukaryote-derived contamination</t>
+  </si>
+  <si>
+    <t>Supplementary Table 9 | Contamination categories identified in the independent post hoc audit</t>
+  </si>
+  <si>
+    <t>Percentages are calculated on a contig-weighted basis. Additional contamination categories represent source-resolved contamination identified during the post hoc audit after primary decontamination. The audit was performed on the 480 Asgard MAGs included in the independently audited dataset. The four complete isolate genomes included in the corresponding phylogenomic analyses were not subject to this MAG-specific contamination audit.</t>
   </si>
 </sst>
 </file>
@@ -394,7 +394,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="17" thickTop="1" x14ac:dyDescent="0.2">
@@ -408,7 +408,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2" s="13"/>
       <c r="F2" s="13"/>
@@ -425,7 +425,7 @@
         <v>4</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>5</v>
@@ -523,9 +523,9 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>

</xml_diff>